<commit_message>
feat: colonne URL (page éditeur, jamais OpenAlex) remplie par scripts/add_urls.py
</commit_message>
<xml_diff>
--- a/data/base_complete.xlsx
+++ b/data/base_complete.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -435,6 +435,7 @@
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,6 +469,11 @@
           <t>University</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -498,6 +504,11 @@
           <t>University of Koudougou</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-031-54235-0_12</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -528,6 +539,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-031-81570-6_10</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -554,6 +570,11 @@
         <v>2024</v>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2024.0150999</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -610,6 +631,11 @@
           <t>University of Koudougou</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/africon51333.2021.9570886</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -640,6 +666,11 @@
           <t>Université Joseph Ki-Zerbo; University of Koudougou; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-319-43696-8_14</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -696,6 +727,11 @@
           <t>University of Koudougou; Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-319-66742-3_8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -726,6 +762,11 @@
           <t>University of Koudougou; Université Ouaga II; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-319-98827-6_36</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -756,6 +797,11 @@
           <t>University of Koudougou; Université Joseph Ki-Zerbo; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-319-43696-8_3</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -786,6 +832,11 @@
           <t>Université Joseph Ki-Zerbo; University of Koudougou</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-030-03405-4_25</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -816,6 +867,11 @@
           <t>Université Joseph Ki-Zerbo; University of Koudougou</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/itnac55475.2022.9998415</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -846,6 +902,11 @@
           <t>Université Joseph Ki-Zerbo; University of Koudougou</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ice3is56585.2022.10010180</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -876,6 +937,11 @@
           <t>Université Joseph Ki-Zerbo; University of Koudougou</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-031-09073-8_17</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -906,6 +972,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4108/eai.11-11-2021.2317973</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -936,6 +1007,11 @@
           <t>University of Koudougou</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2022.01309106</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -966,6 +1042,11 @@
           <t>Université Joseph Ki-Zerbo; Institut Supérieur de l'Informatique et de Gestion</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/ojapps.2022.1212146</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -996,6 +1077,11 @@
           <t>Nazi Boni University; Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/sccic51516.2020.9377330</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1026,6 +1112,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-030-89906-6_61</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1056,6 +1147,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/inc457730.2023.10262859</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1086,6 +1182,11 @@
           <t>Nazi Boni University; Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-031-38333-5_23</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1116,6 +1217,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-981-16-9416-5_59</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1142,6 +1248,11 @@
         <v>2023</v>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.procs.2023.01.397</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1172,6 +1283,11 @@
           <t>Université Joseph Ki-Zerbo; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-030-63329-5_9</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1202,6 +1318,11 @@
           <t>Université Joseph Ki-Zerbo; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-031-34896-9_12</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1232,6 +1353,11 @@
           <t>University of Koudougou; Institut de l'Environnement et Recherches Agricoles</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/jilsa.2022.141001</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1262,6 +1388,11 @@
           <t>University of Koudougou; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/africon55910.2023.10293534</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1292,6 +1423,11 @@
           <t>University of Koudougou</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-031-35883-8_5</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1322,6 +1458,11 @@
           <t>University of Koudougou; Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/icfsp59764.2023.10372941</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1352,6 +1493,11 @@
           <t>Université Joseph Ki-Zerbo; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3233/shti250696</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1382,6 +1528,11 @@
           <t>Centre National de la Recherche Scientifique et Technologique</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5281/zenodo.18272349</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1412,6 +1563,11 @@
           <t>Université Ouaga II</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64388/irev9i8-1714442</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1442,6 +1598,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.62411/jcta.12021</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1472,6 +1633,11 @@
           <t>Institut de Recherche Pour le Développement</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.procs.2025.07.195</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1502,6 +1668,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.23919/icn.2025.0022</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1532,6 +1703,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/jst.2025.151002</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1562,6 +1738,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ictas64866.2025.11155839</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1592,6 +1773,11 @@
           <t>Université Joseph Ki-Zerbo; Université Aube Nouvelle</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/eng.2025.171008</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1622,6 +1808,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/iceeng64546.2025.11031345</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1652,6 +1843,11 @@
           <t>Université Joseph Ki-Zerbo; Université Aube Nouvelle; University of Koudougou</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/wjnse.2025.151001</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1682,6 +1878,11 @@
           <t>Nazi Boni University; Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1117/12.3066050</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1712,6 +1913,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/aiiot65859.2025.11105297</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1742,6 +1948,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/icsc65596.2025.11139942</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1772,6 +1983,11 @@
           <t>University of Koudougou; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/acdsa65407.2025.11166262</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1802,6 +2018,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/acdsa65407.2025.11165890</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1832,6 +2053,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/acdsa65407.2025.11166202</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1862,6 +2088,11 @@
           <t>Université Joseph Ki-Zerbo; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/acdsa65407.2025.11166159</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1892,6 +2123,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/c4d65382.2025.11306472</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1922,6 +2158,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2024.01507135</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1952,6 +2193,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/icabcd62167.2024.10645267</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1982,6 +2228,11 @@
           <t>University of Koudougou</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3659677.3659684</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2012,6 +2263,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/acai63924.2024.10899704</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2042,6 +2298,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/mne3sd63831.2024.10812147</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2072,6 +2333,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://hal.science/hal-04425409</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2102,6 +2368,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35940/ijrte.d8153.13041124</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2132,6 +2403,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/mne3sd63831.2024.10812117</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2162,6 +2438,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/icngn63705.2024.10871579</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2192,6 +2473,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/icecer62944.2024.10920314</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2222,6 +2508,11 @@
           <t>Institut de Recherche Pour le Développement</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/africon55910.2023.10293321</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2252,6 +2543,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/mne3sd57078.2023.10079830</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2282,6 +2578,11 @@
           <t>Université Joseph Ki-Zerbo; Nazi Boni University</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2023.01406136</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2312,6 +2613,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5121/ijnlc.2023.12401</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2342,6 +2648,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.59200/icarti.2023.013</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2372,6 +2683,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.12785/ijcds/140146</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2402,6 +2718,11 @@
           <t>Nazi Boni University; University of Koudougou</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/mne3sd57078.2023.10079800</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2432,6 +2753,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.12785/ijcds/140145</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2462,6 +2788,11 @@
           <t>University of Koudougou</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3604383.3604387</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2492,6 +2823,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/mne3sd53781.2022.9723173</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2522,6 +2858,11 @@
           <t>Nazi Boni University; AFRICSanté; West African Health Organisation; Centre Muraz</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2021.0120374</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2552,6 +2893,11 @@
           <t>University of Koudougou; Université Aube Nouvelle</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/imitec52926.2021.9714675</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2582,6 +2928,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.23919/cisti52073.2021.9476498</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2612,6 +2963,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/besc51023.2020.9348311</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2642,6 +2998,11 @@
           <t>Institut de l'Environnement et Recherches Agricoles</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.knosys.2020.106220</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2672,6 +3033,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/sccic51516.2020.9377331</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2702,6 +3068,11 @@
           <t>Nazi Boni University; Centre Muraz</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2020.0111293</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2732,6 +3103,11 @@
           <t>Nazi Boni University</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ibase-bf48578.2020.9069588</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2762,6 +3138,11 @@
           <t>Global Water Partnership West Africa</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.29121/granthaalayah.v8.i8.2020.1181</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2792,6 +3173,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/isc246665.2019.9071738</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2822,6 +3208,11 @@
           <t>Université Joseph Ki-Zerbo; Université Ouaga II</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5539/cis.v12n3p81</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2852,6 +3243,11 @@
           <t>Institut Supérieur de l'Informatique et de Gestion</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.60713/pist-147610</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2882,6 +3278,11 @@
           <t>Université Ouaga II</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5120/ijca2017915720</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2912,6 +3313,11 @@
           <t>University of Koudougou</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2016.070466</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2942,6 +3348,11 @@
           <t>Nazi Boni University; Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5121/ijdms.2016.8201</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3002,6 +3413,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/jcc.2015.36011</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3032,6 +3448,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/jcc.2015.38005</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3062,6 +3483,11 @@
           <t>Institut de l'Environnement et Recherches Agricoles</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/18756891.2013.818185</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3092,6 +3518,11 @@
           <t>Institut de l'Environnement et Recherches Agricoles</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://hal.science/hal-00811748</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3122,6 +3553,11 @@
           <t>Université Joseph Ki-Zerbo</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/icimp.2009.29</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3150,6 +3586,11 @@
       <c r="F91" s="2" t="inlineStr">
         <is>
           <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-0-387-49690-0_6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: corpus étendu à 116 articles d'informatique burkinabè
</commit_message>
<xml_diff>
--- a/data/base_complete.xlsx
+++ b/data/base_complete.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3594,6 +3594,916 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Document_91</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Software Defined Networks: Strengths, Weaknesses, and Resilience to Failures</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>This article examines the architecture of software-defined networks (SDN) and its implications for the modern management of communications infrastructures. By decoupling the control plane from the data plane, SDN offers increased flexibility and programmability, enabling rapid adaptation to changing user requirements. However, this new approach poses significant challenges in terms of security, fault tolerance, and interoperability. This paper highlights these challenges and explores current strategies to ensure the resilience and reliability of SDN networks in the face of threats and failures. In addition, we analyze the future outlook for SDN and the importance of integrating robust security solutions into these infrastructures.</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Wendnéso Aïda Ouedraogo Rakissaga; Omar Harouna Hamidou; Pegdwindé Justin Kouraogo</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Institut Supérieur de l'Informatique et de Gestion; Université Aube Nouvelle; Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4236/eng.2025.171002</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Document_92</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Preventing DDoS Attacks in SDN Networks: A Model of Defense Against Packet-in Flooding</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>The Software-Defined Networking (SDN) paradigm is increasingly attracting market players due to the centralization of control functions and the physical distinction between the control and data planes. However, it is not immune to disruptions caused by misconfigurations, cyberattacks, or natural disasters. Moreover, the primary benefit of SDN, centralized network control, also makes it highly susceptible to DDoS (Distributed Denial of Service) attacks. As a result, DDoS attacks pose a considerable threat to the security of SDN networks. To address this issue, we focus on a specific type of message known as the 'packet-in.' In SDN network operations, when a switch receives a new packet and does not find a match in its flow table, it requests a forwarding rule from the controller via a packet-in message. We leverage this type of message to propose a solution for preventing DDoS attacks in SDN environments. Several approaches have been explored to counter DDoS attacks in SDN networks, but most involve the controller. This presents two limitations: first, it increases the controller’s workload, which is already heavily utilized in the SDN architecture; second, it is preferable to eliminate the attack at the network’s edge. The proposed solution involves monitoring the number of distinct destinations contacted by a given source within a specific time window, based on the quantity of packet-in messages triggered by that source. If the number of unique destinations exceeds a predefined threshold, the source node is deemed suspicious and placed in quarantine. Through our solution, which enables the identification and blocking of DDoS attacks directly at the data plane, we contribute to reducing the controller’s workload and facilitating rapid decision-making (no need to send a Packet-In to the controller for every suspicious packet).</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Wendnéso Aïda Ouedraogo Rakissaga; Pegdwindé Justin Kouraogo; Tounwendyam Frédéric Ouédraogo</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Université Joseph Ki-Zerbo; University of Koudougou</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/aiiot65859.2025.11105220</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Document_93</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Fakipedia: Building and exploiting an AI model for detecting online fake news in Burkina Faso</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Misinformation poses a significant challenge, especially in developing countries with low literacy rates. The rapid spread on social media, coupled with their lack of robust verification mechanisms, makes distinguishing between credible and false information increasingly difficult. This document outlines our efforts to address this challenge in Burkina Faso using the pre-trained linguistic model CAMEMBERT. Our preliminary results show high performance (up to a 99.34% F1 score) on Fakipedia, suggesting that certain blatant instances of false information can be effectively identified and stopped by automated tools.</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Angelique Sidbewendin Yameogo; Aminata Sabané; Tegawendé François Bissyandé; Rodrique Kafando; Abdoul-Kader Kabore</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://hal.science/hal-04425410</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Document_94</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Design and Implementation of a Knowledge Graph for Integrating Global Health Data Using Neo4j</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Global health research requires the integration of diverse datasets and continuous updates to enable more effective monitoring and interpretation of global health trends. However, traditional tabular datasets often fall short in accommodating multiple datasets with heterogeneous schemas and evolving structures, and they hinder the efficient updating of such datasets once integrated. Graph databases offer a natural solution to these challenges by providing a flexible data structure that can explicitly represent complex relationships and accommodate incremental updates without requiring modifications to existing data. This paper presents an initial attempt to apply graph database technology to global health research by proposing a structured roadmap for constructing a Neo4j-based knowledge graph from heterogeneous data sources. The application of knowledge graphs in global health research enables comprehensive, up-to-date representation of complex datasets, facilitates direct insights into multifaceted relationships, supports multi-perspective analyses, and establishes a foundation for scalable and analytically robust research in the field.</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Yuerui Yan; Ali Sié; Valentin Boudo; Pascal Zabré; Aristide Ouedraogo; Sandra Barteit</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Centre de Recherche en Santé de Nouna</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3233/shti260882</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Document_95</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Design of an Intelligent Chatbot for Assisting Medical Diagnosis Within a Holistic Healthcare Approach in Burkina Faso</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>In low-resource healthcare environments such as Burkina Faso, limited access to medical professionals, combined with sociocultural barriers, creates delays in early diagnosis and care-seeking behavior. This paper presents the design, implementation, and evaluation of a culturally-aware intelligent medical chatbot that supports first-line diagnostic guidance within a holistic healthcare framework integrating physical, psychological, and contextual dimensions. Unlike conventional chatbots relying solely on general-purpose NLP models, the proposed system introduces a hybrid architecture combining rule-based reasoning and a domain-specific natural language processing engine (API G3N35I5) enriched with locally grounded symptom expressions. The system is designed to interpret both biomedical symptoms and culturally encoded expressions of discomfort. A pilot evaluation involving 25 participants demonstrates an average response time of 1.1 seconds, symptom interpretation accuracy of 87%, and user satisfaction of 92%, indicating that culturally-adapted AI systems can significantly improve early health orientation in low-resource contexts.</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Thomas Alassane Ouattara; Wilfried Ange Bérenger Yaro</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3233/shti260803</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Document_96</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Towards a Chatbot for Medical Diagnosis Based on Patient Symptoms</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>The advent of artificial intelligence has positively transformed many areas of our lives, including the medical field. In this article, we propose the development of a medical diagnosis chatbot based on patients' symptoms, using artificial intelligence as an innovative solution. The aim of this tool is to provide doctors with a preliminary diagnosis based on the symptoms presented by patients. Our proposal involves first building models to be used for predicting diseases, and then using a llama-inspired model to generate the medical report and prescription. The chatbot system was implemented using Python, HTML, CSS and JavaScript, with FastAPI for the RESTful API and PostgreSQL for data management. The results highlight the potential of AI to improve healthcare services, especially in areas where resources are limited.</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Kiswendsida Kisito Kaboré; Omar Sawadogo; Yaya Traoré; Julie Thiombiano</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3233/shti240570</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Document_97</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Conception of an Intelligent Chatbot for Creation of an African Virtual Patient</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Medical and paramedical training is still a major issue in Africa, given the growing needs that contrast with the shortage of teachers, hospitals and educational facilities. The aim of the present work is to design an artificial intelligence that enables a virtual patient to hold a conversation with a doctor or a student. To achieve this, we first carried out a literature review on the various approaches to designing artificial intelligence of this type. Next, we selected the tools needed to develop the intelligent model. Finally, we developed and trained our intelligent model to hold a conversation with a healthcare professional during a medical consultation.</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Jonathan Kambire; Seydou Golo Barro; Pascal Staccini</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3233/shti250040</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Document_98</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>New Robust Watermarking Scheme for a Distributed Database with Hyperbolic Structure</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>In this paper we propose a new robust water-marking scheme for medical images stored in a distributed database with a hyperbolic structure. Our approach is to first generate a watermark from the patient information and the statistical parameters of the image. The watermark is then inserted into the image and fragmented before being distributed to different nodes. The repartition is carried out using the hyper-catadioptric projection model in order to guarantee its robustness. The receiver extracts the watermark from the image and look for watermark fragments stored in the nodes before proceeding with a comparison. Simulation results clearly show that any attempt to modify the image or the watermark will be detected. The asynchronous stream cryptography technique has been proposed to restore data in the event of an attack. The implementation of the hyper-catadioptric model enabled us to adapt our watermarking scheme to the structure of the distributed database. Finally, formal analysis and simulations allow us to state that our system is chaotic and therefore robust.</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Boureima Koussoube; Moustapha Bikienga; Telesphore Tiendrebeogo</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University; University of Koudougou</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/icbea66055.2025.00023</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Document_99</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Addressing Challenges in Data Quality and Model Generalization for Malaria Detection</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Malaria remains a significant global health burden, particularly in resource-limited regions where timely and accurate diagnosis is critical to effective treatment and control. Deep Learning (DL) has emerged as a transformative tool for automating malaria detection and it offers high accuracy and scalability. However, the effectiveness of these models is constrained by challenges in data quality and model generalization including imbalanced datasets, limited diversity and annotation variability. These issues reduce diagnostic reliability and hinder real-world applicability. This article provides a comprehensive analysis of these challenges and their implications for malaria detection performance. Key findings highlight the impact of data imbalances which can lead to a 20% drop in F1-score and regional biases which significantly hinder model generalization. Proposed solutions, such as GAN-based augmentation, improved accuracy by 15-20% by generating synthetic data to balance classes and enhance dataset diversity. Domain adaptation techniques, including transfer learning, further improved cross-domain robustness by up to 25% in sensitivity. Additionally, the development of diverse global datasets and collaborative data-sharing frameworks is emphasized as a cornerstone for equitable and reliable malaria diagnostics. The role of explainable AI techniques in improving clinical adoption and trustworthiness is also underscored. By addressing these challenges, this work advances the field of AI-driven malaria detection and provides actionable insights for researchers and practitioners. The proposed solutions aim to support the development of accessible and accurate diagnostic tools, particularly for resource-constrained populations</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Kiswendsida Kisito Kaboré; Désiré Guel</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Université Ouaga II; Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.33140/jsndc.04.03.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Document_100</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Eco-Friendly AI-Based Classification System for Payment Card Support Tickets</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>The payment card industry has revolutionized the way we use and interact with money.The Card Payment Support Department is responsible for customer management, ensuring that bank cards, ATMs, POS terminals, and online stores function properly, allowing users to make transactions with their bank cards anytime and anywhere.The Payment Service Center serves as the first point of contact for customers, and its main challenges include the ability to quickly categorize customer requests, consistently resolve tickets within the SLA (Service Level Agreement), and enhance the user experience.In this paper, we propose a fine-tuned Large Language Model (LLM) to automatically classify incoming customer requests.Our model achieved an average accuracy of 76.74% across 51 categories, using only 3 epochs.The complete code and model are available online.We also developed a web application with Streamlit that leverages our model to predict the category of incoming tickets and automatically assign the request to the correct department when the model's confidence is higher than 40%.</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Metouole Mwinbe Yves Ghislain Somda; Attoumane Tahar; Thierry Kondengar; Rodrique Kafando; Mamadou Ba; Samuel Ouya; Gervais Mendy</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Université Ouaga II</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3719384.3719441</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Document_101</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Detection of Android Malware based on Sequence Alignment of Permissions</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Permissions control accesses to critical resources on Android.Any weaknesses from their exploitation can be of great interest to attackers.Investigation about associations of permissions can reveal some patterns against attacks.In this regards, this paper proposes an approach based on sequence alignment between requested permissions to identify similarities between applications.Permission patterns for malicious and normal samples are determined and exploited to evaluate a similarity score.The nature of an application is obtained based on a threshold, judiciously computed.Experiments have been realized with a dataset of 534 malicious samples (300 training and 234 testing) and 534 normal samples (300 training and 234 testing).Our approach has been able to recognize testing samples (either malware or normal) with an accuracy of 79%, an average precision of 76% and an average recall of 75%.This research reveals that sequence alignment can improve malware detection research.</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Franklin Tchakounté; Albert Djakene Wandala; Yélémou Tiguiane</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.ijcjournal.org/index.php/InternationalJournalOfComputer/article/view/1455</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Document_102</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Towards Blockchain Services For Mobile Money Traceability And Federation</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>This paper discusses a new approach to mobile money, a money transfer solution via mobile phone, which uses accounts associated with SIM (Subscriber Identity Module) identifiers, and which are managed by the Mobile Network Operators (MNOs). The first solution launched in Kenya in 2007, M-PESA is one of the world major mobile money services. Mobile money becomes the new monopoly of MMOs in an economic system where the rate of unbanked adults is very high. Currently in 2019 Orange Money makes nearly 1.5 million transactions per day, which corresponds to a monetary value of nearly 15 billion CFA francs per day. The USSD is the technology at the heart of the Mobile-money transactions. Blockchain, which is the underlying technology of the first crypto currency Bitcoin, has drawn a lot of global attention in recent years. Blockchain does not stop seeing its field of action widen. The field of action of the Blockchain has not yet completed its enlargement. The rate of unbanked is still very high in developing countries; this rate is a factor that does not favor the emergence of the economy. It is necessary to count on the mobile money to skip this obstacle (according to the World Bank) we make here the state of the art on the mobile money and its underlying technologies in the sub-Saharan countries and in Burkina-Faso. We propose a mobile-money solution based on the Blockchain, in order to increase security, trust, and move towards a federation of mobile-money platforms.</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Kodjo Edem Agbezoutsi; Pascal Urien; Toundé Mesmin Dandjinou</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/csnet47905.2019.9108970</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Document_103</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Cloak-Reduce Load Balancing Strategy for Mapreduce</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>The advent of Big Data has seen the emergence of new processing and storage challenges. These challenges are often solved by distributed processing. Distributed systems are inherently dynamic and unstable, so it is realistic to expect that some resources will fail during use. Load balancing and task scheduling is an important step in determining the performance of parallel applications. Hence the need to design load balancing algorithms adapted to grid computing. In this paper, we propose a dynamic and hierarchical load balancing strategy at two levels: Intrascheduler load balancing, in order to avoid the use of the large-scale communication network, and interscheduler load balancing, for a load regulation of our whole system. The strategy allows improving the average response time of CLOAK-Reduce application tasks with minimal communication. We first focus on the three performance indicators, namely response time, process latency and running time of MapReduce tasks.</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Mamadou Diarra; Telesphore Tiendrebeogo</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5121/ijcsit.2021.13403</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Document_104</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Big Data Processing of Cloak-Reduce</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Big Data has introduced the challenge of storing and processing large volumes of data (text, images, and videos). The success of centralised exploitation of massive data on a node is outdated, leading to the emergence of distributed storage, parallel processing and hybrid distributed storage and parallel processing frameworks. The main objective of this paper is to evaluate the load balancing and task allocation strategy of our hybrid distributed storage and parallel processing framework CLOAK-Reduce. To achieve this goal, we first performed a theoretical approach of the architecture and operation of some DHT-MapReduce. Then, we compared the data collected from their load balancing and task allocation strategy by simulation. Finally, the simulation results show that CLOAK-Reduce C5R5 replication provides better load balancing efficiency, MapReduce job submission with 10% churn or no churn.</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Mamadou Diarra; Telesphore Tiendrebeogo</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5121/ijdps.2022.13102</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Document_105</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Big Data Storage System Based on a Distributed Hash Tables System</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>The Big Data is unavoidable considering the place of the digital is the predominant form of communication in the daily life of the consumer. The control of its stakes and the quality its data must be a priority in order not to distort the strategies arising from their treatment in the aim to derive profit. In order to achieve this, a lot of research work has been carried out companies and several platforms created. MapReduce, is one of the enabling technologies, has proven to be applicable to a wide range of fields. However, despite its importance recent work has shown its limitations. And to remedy this, the Distributed Hash Tables (DHT) has been used. Thus, this document not only analyses the and MapReduce implementations and Top-Level Domain (TLD)s in general, but it also provides a description of a model of DHT as well as some guidelines for the planification of the future research.</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Telesphore Tiendrebeogo; Mamadou Diarra</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5121/ijdms.2020.12501</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Document_106</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Big Data Storage based on CAN Protocol</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Big Data refers to huge amounts of heterogeneous data from various traditional and new data sources. This data is constantly changing. However, due to their great heterogeneity, several architectural approaches are proposed to centrally process and analyze the huge amounts of data. A Big Data architecture describes the blueprint of a system that processes a huge amount of data from its storage, processing, analysis and visualization. From one architecture to another, there are advantages and limitations especially in terms of time and processing mode. In our paper, we propose a decentralized architecture based on the peer-to-peer protocol CAN (Content Adressable Network) using image properties associated with SHA-512 keys to secure the data. First, we evaluated the existing Big Data technologies from the architecture to the data storage model. Then, we presented all the conceptual aspects of our architecture and we ended with the evaluation of a symbolic version developed and deployed in a local network.</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Lacine KABRE; Telesphore Tiendrebeogo</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-2688243/v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Document_107</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Android AI Application for Advanced Breast Cancer Detection in Burkina Faso</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>The adaptation of a breast cancer detection platform based on artificial intelligence, designed for use on Android devices, is an initiative driven by the particular challenges faced in Africa, where access to computers is often limited due to their high cost and limited availability, a significant issue in Burkina Faso. It is especially crucial to find tailored and more efficient solutions for healthcare professionals in such environments. This mobile adaptation aims to make this advanced technology more accessible to healthcare professionals across the country, with mobile devices being far more common and accessible, with around 86% coverage in Burkina Faso. Our goal is to simplify the work of pathologists by enabling them to benefit from the advantages of AI for early and accurate breast cancer detection, directly from mobile devices, without requiring expensive infrastructure.</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Seydou Golo Barro; Thomas Alassane Ouattara; Pascal Staccini</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3233/shti250041</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Document_108</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>HoughVG:Hough Transform Toolbox for Straight-Line Detection and Fingerprint Recognition</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>This paper presents HoughVG (Hough transform on Virtual Grid), a toolbox that improves on the Hough transform method, originally developed in 1962, by optimizing it for straight line detection and fingerprint recognition. Drawing on innovative approaches such as the rectangular, triangular, hexagonal and octagonal Hough transforms, as well as the generalized Hough transform, HoughVG significantly improves detection accuracy and processing speed. The toolbox is designed with a modular architecture, offering both sequential and parallelized functions. HoughVG’s test results indicate its potential impact on various fields, from academic research to industrial applications, while taking into account the limitations associated with pattern detection and parameter tuning. • HoughVG (Hough transform on Virtual Grid) is a toolbox that enhances Hough transform. • Toolbox uses different Hough transforms:Hexagonal, Octagonal, Rectangular, Triangular • Toolbox takes into account straight line detection and fingerprint recognition. • Toolbox allows to choose sequential or parallelized functions. • Toolbox is applicable in robotics, medical imaging, security, biometrics.</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Moïse Ouedraogo; Abdoulaye Séré; Cheick Amed Diloma Gabriel Traoré</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.simpa.2024.100709</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Document_109</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Hough Transform based on Object Dual and Pymp Library</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Geometric shape detection in an image is a classical problem that leads to many applications, in cartography to highlight roads in a noisy image, in medical imaging to localize disease in a region and in agronomy to fight against weeds with pesticides. The Hough Transform method contributes effectively to the recognition of digital objects, as straight lines, circles and arbitrary objects. This paper deals with the theoretical comparisons of object dual based on the definition of Standard Hough Transform. It also focuses on parallelism of Hough Transform. A generic pseudo-code algorithm, using the Openmp library for the parallel computing of object dual is proposed in order to improve the execution time. In simulation, a triangular mesh superimposed on the image is implemented with the pymp library in python, in considering threads as inputs to read the image and to update the accumulator. The parallel computing presents reduction of the execution time accordingly to the rate of lit pixels in each virtual object and the number of threads. In perspectives, it will contribute to strenghen the developement of a toolkit for the Hough Transform method.</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Abdoulaye Séré; Moise OUEDRAOGO; Armand Kodjo Atiampo</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.14569/ijacsa.2022.0131084</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Document_110</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Semantic annotation of resources based on ontologies:application to a knowledge sharing platform on meningitis</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Semantic annotation of resources with ontologies plays a decisive role for semantic search, interoperability and data integration. In this paper, we focus on semi-automated web page annotation for a meningitis knowledge sharing platform. This web page annotation refers to the introduction of categories on a page or a set of tags on a page. Thus, we present a semantic web page annotation approach based on the use of an ontology. In this proposal, ontology is used to determine the categories on the web page. Our method extracts the relevant terms called keywords in the page to annotate. Our strategy for identifying the categories focus on ontology's concepts similarity with each keyword. The tags are identified among the keywords that are not mapped to the ontology's concepts. The results of simulation indicate the approach is feasible for practical use in semantic annotation of a new web page.</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Julie Thiombiano; Yaya Traoré; Sadouanouan Malo; Patrice Koassa; Oumarou Sié</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/sccic51516.2020.9377332</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Document_111</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Towards an Architecture for the Interoperability of Hospital Information Systems in Burkina Faso</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>The successful introduction of ICTs into medical practice is a key factor in improving the performance of any health system for both patients and healthcare professionals. In Burkina Faso, many hospital information systems (HIS) have been developed and are already widely used in large health centers with proven efficiency. To improve the quality of patient care, these hospital information systems should exchange information. Interoperability is one of the privileged ways to improve the integration of different systems because nowadays a HIS is no longer just a single monolithic software system, which is run on a single machine. This paper presents a semantic interoperability architecture, which is based on a mediation approach. The mediator implements local domain ontologies for each HIS, a knowledge base, and a referential ontology which is used as a semantic repository and web services.</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Tapsoba Lydie Simone; Yaya Traoré; Sadouanouan Malo</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University; Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3233/shti200518</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Document_112</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Fault-Tolerant Routing protocol for Ad Hoc Networks</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Wireless Ad Hoc networks are faulty networks because they are usually deployed in harsh environment. So, routing protocols in Ad Hoc networks must be fault aware to reduce loosing data because of link or node failure. A fault- tolerant routing is a robust mechanism that allows routing protocols to react to failures that might occur in the network. Most importantly, they allow the network to continue to operate as expected without failures.In this paper, we propose a fault tolerant hop count based routing protocol (F-Hopcount) for WSNs that is able to cope with random node failures with very little impacting on the overall network performances. We evaluated our proposal using Cooja simulator and compared it to the standard hop count rountig protocol. Results show that our contribution supports node failures very well in the studied scenarios with very little impact on the network performances.</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Mesmin Dandjinou; Hamadoun Tall; Tiguiane Yélémou</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ibase-bf48578.2020.9069590</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Document_113</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>A SDN based approach to improve energy consumption in wireless ad hoc network</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Ad-hoc wireless networks are increasingly being used in communications especially in surveillance situations in unfriendly environments. Energy management problem of these communicating autonomous nodes is a major handicap especially for countries with limited financial resources. Indeed, the lifespan of this type of network is that of a few nodes. In this article, we propose the use of Software-Defined Networking (SDN) technology to optimize energy consumption in these nodes. In our approach, establishment and maintenance of path is provided by a controller. Nodes focus on packet switching. This approach is implemented in the well known reactive routing protocol, Ad hoc On-demand Distance Vector (AODV). Analysis of performances of this new protocol, SDN based AODV (S-AODV), that we propose, shows that, comparing with the standard AODV, we significantly improve nodes energy consumption and thus the lifespan of these types of networks, routing load and path establishment delay.</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Mahamadi Boulou; Tiguiane Yélémou; Pegdwindé Justin Kouraogo; Doda Afoussatou Rollande; Hatem Ben Sta</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University; Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/isc246665.2019.9071739</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Document_114</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Neighbor Discovery Algorithms in a Star WSN: Switched beam antenna vs omnidirectional antenna at the Sink</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>One of the key element in performance measurement for a neighbor discovery algorithm with switched beam antennas is how long it takes to discover the neighbors given that nodes do not have any prior knowledge about their neighbors. An impression we may have in neighbor discovery is that algorithms based on directional antennas takes longer time for a node to discover all its neighbors than those entirely based on omnidirectional antennas. We propose two neighbor discovery schemes, one is based on time slotting and the other on the well known CSMA/CA unslotted version. We evaluate the time that the sink needs to discover its neighbors when it is equipped with a switched beam antenna, and when it uses an omnidirectional antenna. Through our simulation results, we show that when neighbor discovery algorithms based on directional antennas are correctly designed, they achieve the same order of performance in terms of time needed by the sink to discover all its neighbors as those based on omnidirectional antennas. Our simulation results also show that when using a switched beam antenna and CSMA/CA algorithm for medium access at the sink, the discovery delay is higher.</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>Guerezuin Der Sylvestre Sidibe; Hamadoun Tall; Marie-Françoise Servajean; Michel Misson</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.23919/pemwn47208.2019.8986963</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Document_115</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Distributed E-learning System using an Hybrid P2P-based Content Addressable Network Architecture</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>We have developed a distributed asynchronous web-based training system.In order to improve the scalability and robustness of this system, all the content and a function are realized on mobile agents.These agents are distributed to computers, and they can use a Peer to Peer network that modifies the DHT Content Addressable Network (CAN).In this system, all computers offer the function and exercise by themselves.However, the system that all computers do the same behavior is not realistic.In this paper, we present an e-learning system composed of computers with different types of participation as a solution to this problem.Activating computers of different types of participation will improve the convenience of the system.</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>Telesphore Tiendrebeogo; Kabre Laciné</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Nazi Boni University; Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5121/ijdps.2020.11501</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Document_116</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>A Lay User Explainable Food Recommendation System Based on Hybrid Feature Importance Extraction and Large Language Models</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Large Language Models (LLM) have experienced strong development in recent years, with varied applications. This paper uses LLMs to develop a post-hoc process that provides more elaborated explanations of the results of food recommendation systems. By combining LLM with a hybrid extraction of key variables using SHAP, we obtain dynamic, convincing and more comprehensive explanations to lay user, compared to those in the literature. This approach enhances user trust and transparency by making complex recommendation outcomes easier to understand for a lay user.</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Melissa Tessa; Diderot D. Cidjeu; Rachele Carli; Sarah Abchiche; Ahmad Aldarwish; Igor Tchappi; Amro Najjar</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Institut de Recherche Pour le Développement</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.procs.2026.04.093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(auteurs): corrige le nom tronque "Franklin Tchakount"
Document_64 et Document_66 : "Franklin Tchakount" (accent detache ou
manquant, extraction PDF) devient "Franklin Tchakounte", comme dans
Document_101. Seules ces deux cellules Authors sont modifiees (verifie par
comparaison cellule a cellule de tout le classeur).

L'alias fusion devenu inutile (plus aucune forme tronquee dans la base) est
retire de data/author_aliases.txt, sinon le demarrage echoue (nom absent de
la base). Tests recalcules sur la base reelle : le groupe Tchakount* sort de
EXPECTED_GROUPS (fusion automatique, sans alias) et le compte sans alias
passe de 186 a 185.
</commit_message>
<xml_diff>
--- a/data/base_complete.xlsx
+++ b/data/base_complete.xlsx
@@ -2672,7 +2672,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Benjamin Savoudsou; Blaise Omer Yenké; Tiguiane Yélémou; Marcellin Atemkeng; Franklin Tchakount ́</t>
+          <t>Benjamin Savoudsou; Blaise Omer Yenké; Tiguiane Yélémou; Marcellin Atemkeng; Franklin Tchakounté</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Franklin Tchakount; Jean Louis Ebongue Kedieng Fendji; Raıssa Manfouo; Didier Bassol; Marcellin Atemkeng</t>
+          <t>Franklin Tchakounté; Jean Louis Ebongue Kedieng Fendji; Raıssa Manfouo; Didier Bassol; Marcellin Atemkeng</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
@@ -3381,6 +3381,11 @@
       <c r="F85" s="2" t="inlineStr">
         <is>
           <t>Université Joseph Ki-Zerbo</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>http://article.sapub.org/10.5923.j.ijit.20160501.03.html</t>
         </is>
       </c>
     </row>

</xml_diff>